<commit_message>
WIP: local changes before switching to collaborator branch
</commit_message>
<xml_diff>
--- a/job_description.xlsx
+++ b/job_description.xlsx
@@ -37,22 +37,22 @@
     <t>Company_name</t>
   </si>
   <si>
-    <t>Machine Learning Intern</t>
-  </si>
-  <si>
-    <t>Currently pursuing or completed a degree in Computer Science, Mathematics, Statistics, or related field</t>
+    <t>Data Science &amp; Engineering Intern</t>
+  </si>
+  <si>
+    <t>Graduate (UG / PG) in Sales and Marketing or Retail management. or Engineering. MBA in Sales and Marketing would be an advantage</t>
   </si>
   <si>
     <t>India</t>
   </si>
   <si>
-    <t>Computer Science and Algorithms skills, Deep Learning and Machine Learning skills, Statistics knowledge, Understanding of neural networks and ensembles, Strong problem-solving skills, Ability to work collaboratively in a team environment, Experience with Python, TensorFlow, or other relevant tools</t>
-  </si>
-  <si>
-    <t>Full-time</t>
-  </si>
-  <si>
-    <t>Shodh AI</t>
+    <t>Python (pandas, NumPy, scikit-learn, etc.), Data engineering and pipeline design, Data cleaning and preprocessing, ML modeling (supervised and unsupervised techniques), Data visualization (Matplotlib, Seaborn, Plotly, or similar), Fluent English Communication Skills (Oral, Written &amp; Presentation), Excellent Spoken &amp; written communication skills in English, and any 1 local language, Good Understanding about Lead Research, Lead Gathering, sales Forecasting in Software, SaaS, Internet or Application based companies</t>
+  </si>
+  <si>
+    <t>Internship</t>
+  </si>
+  <si>
+    <t>Razonica</t>
   </si>
 </sst>
 </file>
@@ -447,7 +447,7 @@
         <v>9</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
book slots and hr panel updated
</commit_message>
<xml_diff>
--- a/job_description.xlsx
+++ b/job_description.xlsx
@@ -37,22 +37,22 @@
     <t>Company_name</t>
   </si>
   <si>
-    <t>Data Science &amp; Engineering Intern</t>
-  </si>
-  <si>
-    <t>Graduate (UG / PG) in Sales and Marketing or Retail management. or Engineering. MBA in Sales and Marketing would be an advantage</t>
-  </si>
-  <si>
-    <t>India</t>
-  </si>
-  <si>
-    <t>Python (pandas, NumPy, scikit-learn, etc.), Data engineering and pipeline design, Data cleaning and preprocessing, ML modeling (supervised and unsupervised techniques), Data visualization (Matplotlib, Seaborn, Plotly, or similar), Fluent English Communication Skills (Oral, Written &amp; Presentation), Excellent Spoken &amp; written communication skills in English, and any 1 local language, Good Understanding about Lead Research, Lead Gathering, sales Forecasting in Software, SaaS, Internet or Application based companies</t>
-  </si>
-  <si>
-    <t>Internship</t>
-  </si>
-  <si>
-    <t>Razonica</t>
+    <t>AI/ML Engineer</t>
+  </si>
+  <si>
+    <t>Bachelor's or Master's degree in Computer Science, Artificial Intelligence, Machine Learning, Data Science, or a closely related quantitative field.</t>
+  </si>
+  <si>
+    <t>Bengaluru, Karnataka, India</t>
+  </si>
+  <si>
+    <t>Python, Pandas, NumPy, Scikit-learn, TensorFlow, PyTorch, Keras, NLP, Computer Vision</t>
+  </si>
+  <si>
+    <t>Full-time</t>
+  </si>
+  <si>
+    <t>Abstrabit Technologies</t>
   </si>
 </sst>
 </file>
@@ -447,7 +447,7 @@
         <v>9</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
updated UI and functions
</commit_message>
<xml_diff>
--- a/job_description.xlsx
+++ b/job_description.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>job_title</t>
   </si>
@@ -37,22 +37,19 @@
     <t>Company_name</t>
   </si>
   <si>
-    <t>Internship AI</t>
-  </si>
-  <si>
-    <t>Engg. background with exposure to Machine Learning &amp; Deep Learning, Artificial Intelligence</t>
-  </si>
-  <si>
-    <t>Bengaluru, Karnataka, India</t>
-  </si>
-  <si>
-    <t>Python, Machine Learning Frameworks like Tensorflow/PyTorch, Network Graph Visualization techniques, Compressible Flow Aerodynamics</t>
+    <t>Data Science Internship in Chennai</t>
+  </si>
+  <si>
+    <t>Chennai, Tamil Nadu, India</t>
+  </si>
+  <si>
+    <t>Artificial intelligence, Python, SQL, Data Analytics, Machine Learning, Data Science, Natural Language Processing (NLP), Deep Learning</t>
   </si>
   <si>
     <t>Internship</t>
   </si>
   <si>
-    <t>Airbus</t>
+    <t>Approlabs</t>
   </si>
 </sst>
 </file>
@@ -440,23 +437,20 @@
       <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>